<commit_message>
Fix mapClimateType to handle Climate Control and Wine climate types
CLIMATE CONTROL/Climate Controlled (720 units) now correctly maps to A
instead of NC. Wine (241 units) now correctly maps to RF instead of NC.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/temp/UnitsTypeDescriptionSummary.xlsx
+++ b/temp/UnitsTypeDescriptionSummary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://extraspace-my.sharepoint.com/personal/louisver_extraspaceasia_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5883" documentId="8_{17EABA81-4A6B-4275-917A-D9BE496B5424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E349D22B-A653-4616-B4C9-A2B64DDFF2C3}"/>
+  <xr:revisionPtr revIDLastSave="5902" documentId="8_{17EABA81-4A6B-4275-917A-D9BE496B5424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65FB9F43-61D4-43A3-B5DD-47A56081A47D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,6 +58,7 @@
     <definedName name="TextRefCopy201">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -78,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2672" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2672" uniqueCount="372">
   <si>
     <t>Internal Name</t>
   </si>
@@ -1253,6 +1254,21 @@
   </si>
   <si>
     <t>Extra Space - Banpo</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>RF</t>
+  </si>
+  <si>
+    <t>A / Premium</t>
+  </si>
+  <si>
+    <t>A / Executive</t>
   </si>
 </sst>
 </file>
@@ -2948,6 +2964,37 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2990,37 +3037,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3305,7 +3321,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="656" row="3">
+  <wetp:taskpane dockstate="right" visibility="1" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -3443,33 +3459,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="179" t="s">
+      <c r="B1" s="190" t="s">
         <v>178</v>
       </c>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
+      <c r="C1" s="190"/>
+      <c r="D1" s="190"/>
+      <c r="E1" s="190"/>
+      <c r="F1" s="190"/>
+      <c r="G1" s="190"/>
+      <c r="H1" s="190"/>
+      <c r="I1" s="190"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="168" t="s">
+      <c r="A2" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="171" t="s">
+      <c r="C2" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="172"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="177" t="s">
+      <c r="D2" s="183"/>
+      <c r="E2" s="184"/>
+      <c r="F2" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="177" t="s">
+      <c r="G2" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H2" s="53" t="s">
@@ -3480,13 +3496,13 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="169"/>
-      <c r="B3" s="169"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
+      <c r="A3" s="180"/>
+      <c r="B3" s="180"/>
+      <c r="C3" s="185"/>
+      <c r="D3" s="186"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
       <c r="H3" s="52" t="s">
         <v>7</v>
       </c>
@@ -3655,31 +3671,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -3690,13 +3706,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -4060,56 +4076,56 @@
       </c>
     </row>
     <row r="20" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="182" t="s">
+      <c r="A20" s="168" t="s">
         <v>111</v>
       </c>
-      <c r="B20" s="183">
-        <v>14</v>
-      </c>
-      <c r="C20" s="184">
+      <c r="B20" s="169">
+        <v>14</v>
+      </c>
+      <c r="C20" s="170">
         <v>27001</v>
       </c>
-      <c r="D20" s="184" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="185">
+      <c r="D20" s="170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="171">
         <v>27032</v>
       </c>
-      <c r="F20" s="186"/>
-      <c r="G20" s="187" t="s">
+      <c r="F20" s="172"/>
+      <c r="G20" s="173" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="188" t="s">
-        <v>14</v>
-      </c>
-      <c r="I20" s="189" t="s">
+      <c r="H20" s="174" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" s="175" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="182" t="s">
+      <c r="A21" s="168" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="183">
+      <c r="B21" s="169">
         <v>15</v>
       </c>
-      <c r="C21" s="184">
+      <c r="C21" s="170">
         <v>28001</v>
       </c>
-      <c r="D21" s="184" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="185">
+      <c r="D21" s="170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="171">
         <v>28013</v>
       </c>
-      <c r="F21" s="186"/>
-      <c r="G21" s="187" t="s">
+      <c r="F21" s="172"/>
+      <c r="G21" s="173" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="188" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21" s="189" t="s">
+      <c r="H21" s="174" t="s">
+        <v>14</v>
+      </c>
+      <c r="I21" s="175" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4708,31 +4724,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>180</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -4743,13 +4759,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -5361,31 +5377,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>181</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -5396,13 +5412,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -5577,29 +5593,29 @@
       </c>
     </row>
     <row r="13" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="182" t="s">
+      <c r="A13" s="168" t="s">
         <v>136</v>
       </c>
-      <c r="B13" s="183">
+      <c r="B13" s="169">
         <v>7</v>
       </c>
-      <c r="C13" s="184">
+      <c r="C13" s="170">
         <v>2200</v>
       </c>
-      <c r="D13" s="184" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="185">
+      <c r="D13" s="170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="171">
         <v>2295</v>
       </c>
-      <c r="F13" s="186"/>
-      <c r="G13" s="187" t="s">
+      <c r="F13" s="172"/>
+      <c r="G13" s="173" t="s">
         <v>127</v>
       </c>
-      <c r="H13" s="188" t="s">
+      <c r="H13" s="174" t="s">
         <v>13</v>
       </c>
-      <c r="I13" s="188" t="s">
+      <c r="I13" s="174" t="s">
         <v>14</v>
       </c>
     </row>
@@ -5685,29 +5701,29 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="182" t="s">
+      <c r="A17" s="168" t="s">
         <v>136</v>
       </c>
-      <c r="B17" s="183">
+      <c r="B17" s="169">
         <v>11</v>
       </c>
-      <c r="C17" s="184">
+      <c r="C17" s="170">
         <v>2000</v>
       </c>
-      <c r="D17" s="184" t="s">
+      <c r="D17" s="170" t="s">
         <v>182</v>
       </c>
-      <c r="E17" s="185">
+      <c r="E17" s="171">
         <v>2303</v>
       </c>
-      <c r="F17" s="186"/>
-      <c r="G17" s="187" t="s">
+      <c r="F17" s="172"/>
+      <c r="G17" s="173" t="s">
         <v>150</v>
       </c>
-      <c r="H17" s="188" t="s">
-        <v>14</v>
-      </c>
-      <c r="I17" s="189" t="s">
+      <c r="H17" s="174" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="175" t="s">
         <v>14</v>
       </c>
     </row>
@@ -5818,31 +5834,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>184</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -5853,13 +5869,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -6001,31 +6017,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>185</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -6036,13 +6052,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -6321,32 +6337,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>201</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -6357,13 +6373,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -6564,32 +6580,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>207</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -6600,13 +6616,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -6780,32 +6796,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>208</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -6816,13 +6832,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -7003,32 +7019,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>209</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -7039,13 +7055,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -7662,32 +7678,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>211</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -7698,13 +7714,13 @@
       </c>
     </row>
     <row r="6" spans="1:11" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -7900,32 +7916,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>212</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -7936,13 +7952,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -8123,32 +8139,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="181" t="s">
+      <c r="B3" s="192" t="s">
         <v>213</v>
       </c>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -8159,13 +8175,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -8346,32 +8362,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>221</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -8382,13 +8398,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -8703,32 +8719,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -8739,13 +8755,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -8990,32 +9006,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>233</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -9026,13 +9042,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -9432,32 +9448,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>248</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -9468,13 +9484,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -9701,7 +9717,7 @@
     <col min="5" max="5" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" customWidth="1"/>
     <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -9772,7 +9788,7 @@
       </c>
       <c r="G5" s="75"/>
       <c r="H5" s="75" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I5" s="76" t="s">
         <v>13</v>
@@ -9803,7 +9819,7 @@
       </c>
       <c r="G6" s="62"/>
       <c r="H6" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I6" s="65" t="s">
         <v>14</v>
@@ -9834,7 +9850,7 @@
       </c>
       <c r="G7" s="62"/>
       <c r="H7" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I7" s="65" t="s">
         <v>14</v>
@@ -9865,7 +9881,7 @@
       </c>
       <c r="G8" s="62"/>
       <c r="H8" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I8" s="65" t="s">
         <v>14</v>
@@ -9896,7 +9912,7 @@
       </c>
       <c r="G9" s="62"/>
       <c r="H9" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I9" s="65" t="s">
         <v>14</v>
@@ -9927,7 +9943,7 @@
       </c>
       <c r="G10" s="62"/>
       <c r="H10" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I10" s="65" t="s">
         <v>13</v>
@@ -9958,7 +9974,7 @@
       </c>
       <c r="G11" s="62"/>
       <c r="H11" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I11" s="65" t="s">
         <v>14</v>
@@ -9989,7 +10005,7 @@
       </c>
       <c r="G12" s="62"/>
       <c r="H12" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I12" s="65" t="s">
         <v>13</v>
@@ -10020,7 +10036,7 @@
       </c>
       <c r="G13" s="62"/>
       <c r="H13" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I13" s="65" t="s">
         <v>13</v>
@@ -10051,7 +10067,7 @@
       </c>
       <c r="G14" s="62"/>
       <c r="H14" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I14" s="65" t="s">
         <v>14</v>
@@ -10082,7 +10098,7 @@
       </c>
       <c r="G15" s="62"/>
       <c r="H15" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I15" s="65" t="s">
         <v>14</v>
@@ -10115,7 +10131,7 @@
         <v>31</v>
       </c>
       <c r="H16" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I16" s="65" t="s">
         <v>14</v>
@@ -10146,7 +10162,7 @@
       </c>
       <c r="G17" s="62"/>
       <c r="H17" s="62" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
       <c r="I17" s="65" t="s">
         <v>14</v>
@@ -10177,7 +10193,7 @@
       </c>
       <c r="G18" s="62"/>
       <c r="H18" s="62" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
       <c r="I18" s="65" t="s">
         <v>14</v>
@@ -10208,7 +10224,7 @@
       </c>
       <c r="G19" s="62"/>
       <c r="H19" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I19" s="65" t="s">
         <v>14</v>
@@ -10239,7 +10255,7 @@
       </c>
       <c r="G20" s="62"/>
       <c r="H20" s="62" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
       <c r="I20" s="65" t="s">
         <v>14</v>
@@ -10270,7 +10286,7 @@
       </c>
       <c r="G21" s="62"/>
       <c r="H21" s="62" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
       <c r="I21" s="65" t="s">
         <v>14</v>
@@ -10301,7 +10317,7 @@
       </c>
       <c r="G22" s="62"/>
       <c r="H22" s="62" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
       <c r="I22" s="65" t="s">
         <v>14</v>
@@ -10332,7 +10348,7 @@
       </c>
       <c r="G23" s="62"/>
       <c r="H23" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I23" s="65" t="s">
         <v>14</v>
@@ -10365,7 +10381,7 @@
         <v>31</v>
       </c>
       <c r="H24" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I24" s="65" t="s">
         <v>14</v>
@@ -10396,7 +10412,7 @@
       </c>
       <c r="G25" s="62"/>
       <c r="H25" s="62" t="s">
-        <v>49</v>
+        <v>368</v>
       </c>
       <c r="I25" s="65" t="s">
         <v>14</v>
@@ -10427,7 +10443,7 @@
       </c>
       <c r="G26" s="62"/>
       <c r="H26" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I26" s="65" t="s">
         <v>14</v>
@@ -10458,7 +10474,7 @@
       </c>
       <c r="G27" s="62"/>
       <c r="H27" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I27" s="65" t="s">
         <v>14</v>
@@ -10491,7 +10507,7 @@
         <v>31</v>
       </c>
       <c r="H28" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I28" s="65" t="s">
         <v>14</v>
@@ -10522,7 +10538,7 @@
       </c>
       <c r="G29" s="62"/>
       <c r="H29" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I29" s="65" t="s">
         <v>14</v>
@@ -10555,7 +10571,7 @@
         <v>31</v>
       </c>
       <c r="H30" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I30" s="65" t="s">
         <v>14</v>
@@ -10586,7 +10602,7 @@
       </c>
       <c r="G31" s="62"/>
       <c r="H31" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I31" s="65" t="s">
         <v>14</v>
@@ -10617,7 +10633,7 @@
       </c>
       <c r="G32" s="62"/>
       <c r="H32" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I32" s="65" t="s">
         <v>14</v>
@@ -10648,7 +10664,7 @@
       </c>
       <c r="G33" s="62"/>
       <c r="H33" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I33" s="65" t="s">
         <v>14</v>
@@ -10681,7 +10697,7 @@
         <v>31</v>
       </c>
       <c r="H34" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I34" s="65" t="s">
         <v>14</v>
@@ -10712,7 +10728,7 @@
       </c>
       <c r="G35" s="62"/>
       <c r="H35" s="62" t="s">
-        <v>49</v>
+        <v>368</v>
       </c>
       <c r="I35" s="65" t="s">
         <v>14</v>
@@ -10743,7 +10759,7 @@
       </c>
       <c r="G36" s="62"/>
       <c r="H36" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I36" s="65" t="s">
         <v>14</v>
@@ -10774,7 +10790,7 @@
       </c>
       <c r="G37" s="62"/>
       <c r="H37" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I37" s="65" t="s">
         <v>14</v>
@@ -10807,7 +10823,7 @@
         <v>31</v>
       </c>
       <c r="H38" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I38" s="65" t="s">
         <v>14</v>
@@ -10840,7 +10856,7 @@
         <v>72</v>
       </c>
       <c r="H39" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I39" s="65" t="s">
         <v>74</v>
@@ -10871,7 +10887,7 @@
       </c>
       <c r="G40" s="62"/>
       <c r="H40" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I40" s="65" t="s">
         <v>74</v>
@@ -10904,7 +10920,7 @@
         <v>72</v>
       </c>
       <c r="H41" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I41" s="65" t="s">
         <v>74</v>
@@ -10935,7 +10951,7 @@
       </c>
       <c r="G42" s="62"/>
       <c r="H42" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I42" s="65" t="s">
         <v>75</v>
@@ -10966,7 +10982,7 @@
       </c>
       <c r="G43" s="62"/>
       <c r="H43" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I43" s="65" t="s">
         <v>75</v>
@@ -10997,7 +11013,7 @@
       </c>
       <c r="G44" s="62"/>
       <c r="H44" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I44" s="65" t="s">
         <v>74</v>
@@ -11028,7 +11044,7 @@
       </c>
       <c r="G45" s="62"/>
       <c r="H45" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I45" s="65" t="s">
         <v>75</v>
@@ -11059,7 +11075,7 @@
       </c>
       <c r="G46" s="62"/>
       <c r="H46" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I46" s="65" t="s">
         <v>75</v>
@@ -11090,7 +11106,7 @@
       </c>
       <c r="G47" s="62"/>
       <c r="H47" s="62" t="s">
-        <v>93</v>
+        <v>369</v>
       </c>
       <c r="I47" s="65" t="s">
         <v>74</v>
@@ -11121,7 +11137,7 @@
       </c>
       <c r="G48" s="62"/>
       <c r="H48" s="62" t="s">
-        <v>93</v>
+        <v>369</v>
       </c>
       <c r="I48" s="65" t="s">
         <v>74</v>
@@ -11152,7 +11168,7 @@
       </c>
       <c r="G49" s="62"/>
       <c r="H49" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I49" s="65" t="s">
         <v>74</v>
@@ -11181,7 +11197,7 @@
       </c>
       <c r="G50" s="62"/>
       <c r="H50" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I50" s="65" t="s">
         <v>74</v>
@@ -11210,7 +11226,7 @@
       </c>
       <c r="G51" s="62"/>
       <c r="H51" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I51" s="65" t="s">
         <v>74</v>
@@ -11239,7 +11255,7 @@
       </c>
       <c r="G52" s="62"/>
       <c r="H52" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I52" s="65" t="s">
         <v>74</v>
@@ -11268,7 +11284,7 @@
       </c>
       <c r="G53" s="62"/>
       <c r="H53" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I53" s="65" t="s">
         <v>74</v>
@@ -11297,7 +11313,7 @@
       </c>
       <c r="G54" s="62"/>
       <c r="H54" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I54" s="65" t="s">
         <v>74</v>
@@ -11326,7 +11342,7 @@
       </c>
       <c r="G55" s="62"/>
       <c r="H55" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I55" s="65" t="s">
         <v>74</v>
@@ -11355,7 +11371,7 @@
       </c>
       <c r="G56" s="62"/>
       <c r="H56" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I56" s="65" t="s">
         <v>74</v>
@@ -11384,7 +11400,7 @@
       </c>
       <c r="G57" s="62"/>
       <c r="H57" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I57" s="65" t="s">
         <v>74</v>
@@ -11413,7 +11429,7 @@
       </c>
       <c r="G58" s="62"/>
       <c r="H58" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I58" s="65" t="s">
         <v>74</v>
@@ -11442,7 +11458,7 @@
       </c>
       <c r="G59" s="62"/>
       <c r="H59" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I59" s="65" t="s">
         <v>74</v>
@@ -11471,7 +11487,7 @@
       </c>
       <c r="G60" s="62"/>
       <c r="H60" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I60" s="65" t="s">
         <v>74</v>
@@ -11500,7 +11516,7 @@
       </c>
       <c r="G61" s="62"/>
       <c r="H61" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I61" s="65" t="s">
         <v>74</v>
@@ -11529,7 +11545,7 @@
       </c>
       <c r="G62" s="62"/>
       <c r="H62" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I62" s="65" t="s">
         <v>74</v>
@@ -11558,7 +11574,7 @@
       </c>
       <c r="G63" s="62"/>
       <c r="H63" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I63" s="65" t="s">
         <v>74</v>
@@ -11587,7 +11603,7 @@
       </c>
       <c r="G64" s="62"/>
       <c r="H64" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I64" s="65" t="s">
         <v>74</v>
@@ -11616,7 +11632,7 @@
       </c>
       <c r="G65" s="62"/>
       <c r="H65" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I65" s="65" t="s">
         <v>74</v>
@@ -11645,7 +11661,7 @@
       </c>
       <c r="G66" s="62"/>
       <c r="H66" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I66" s="65" t="s">
         <v>74</v>
@@ -11674,7 +11690,7 @@
       </c>
       <c r="G67" s="62"/>
       <c r="H67" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I67" s="65" t="s">
         <v>74</v>
@@ -11703,7 +11719,7 @@
       </c>
       <c r="G68" s="62"/>
       <c r="H68" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I68" s="65" t="s">
         <v>74</v>
@@ -11732,7 +11748,7 @@
       </c>
       <c r="G69" s="62"/>
       <c r="H69" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I69" s="65" t="s">
         <v>74</v>
@@ -11761,7 +11777,7 @@
       </c>
       <c r="G70" s="62"/>
       <c r="H70" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I70" s="65" t="s">
         <v>74</v>
@@ -11790,7 +11806,7 @@
       </c>
       <c r="G71" s="62"/>
       <c r="H71" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I71" s="65" t="s">
         <v>74</v>
@@ -11819,7 +11835,7 @@
       </c>
       <c r="G72" s="62"/>
       <c r="H72" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I72" s="65" t="s">
         <v>74</v>
@@ -11848,7 +11864,7 @@
       </c>
       <c r="G73" s="62"/>
       <c r="H73" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I73" s="65" t="s">
         <v>74</v>
@@ -11877,7 +11893,7 @@
       </c>
       <c r="G74" s="62"/>
       <c r="H74" s="62" t="s">
-        <v>97</v>
+        <v>367</v>
       </c>
       <c r="I74" s="65" t="s">
         <v>74</v>
@@ -11906,7 +11922,7 @@
       </c>
       <c r="G75" s="62"/>
       <c r="H75" s="62" t="s">
-        <v>73</v>
+        <v>368</v>
       </c>
       <c r="I75" s="65" t="s">
         <v>74</v>
@@ -11937,7 +11953,7 @@
         <v>112</v>
       </c>
       <c r="H76" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I76" s="65" t="s">
         <v>14</v>
@@ -11966,7 +11982,7 @@
       </c>
       <c r="G77" s="62"/>
       <c r="H77" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I77" s="65" t="s">
         <v>14</v>
@@ -11995,7 +12011,7 @@
       </c>
       <c r="G78" s="62"/>
       <c r="H78" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I78" s="65" t="s">
         <v>14</v>
@@ -12024,7 +12040,7 @@
       </c>
       <c r="G79" s="62"/>
       <c r="H79" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I79" s="65" t="s">
         <v>14</v>
@@ -12053,7 +12069,7 @@
       </c>
       <c r="G80" s="62"/>
       <c r="H80" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I80" s="65" t="s">
         <v>14</v>
@@ -12082,7 +12098,7 @@
       </c>
       <c r="G81" s="62"/>
       <c r="H81" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I81" s="65" t="s">
         <v>14</v>
@@ -12111,7 +12127,7 @@
       </c>
       <c r="G82" s="62"/>
       <c r="H82" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I82" s="65" t="s">
         <v>14</v>
@@ -12142,7 +12158,7 @@
         <v>31</v>
       </c>
       <c r="H83" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I83" s="65" t="s">
         <v>14</v>
@@ -12171,7 +12187,7 @@
       </c>
       <c r="G84" s="62"/>
       <c r="H84" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I84" s="65" t="s">
         <v>14</v>
@@ -12200,7 +12216,7 @@
       </c>
       <c r="G85" s="62"/>
       <c r="H85" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I85" s="65" t="s">
         <v>14</v>
@@ -12229,7 +12245,7 @@
       </c>
       <c r="G86" s="62"/>
       <c r="H86" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I86" s="65" t="s">
         <v>14</v>
@@ -12258,7 +12274,7 @@
       </c>
       <c r="G87" s="62"/>
       <c r="H87" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I87" s="65" t="s">
         <v>14</v>
@@ -12287,7 +12303,7 @@
       </c>
       <c r="G88" s="62"/>
       <c r="H88" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I88" s="65" t="s">
         <v>14</v>
@@ -12316,7 +12332,7 @@
       </c>
       <c r="G89" s="62"/>
       <c r="H89" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I89" s="65" t="s">
         <v>14</v>
@@ -12334,7 +12350,7 @@
       <c r="C90" s="65">
         <v>15</v>
       </c>
-      <c r="D90" s="192">
+      <c r="D90" s="178">
         <v>28001</v>
       </c>
       <c r="E90" s="65" t="s">
@@ -12345,7 +12361,7 @@
       </c>
       <c r="G90" s="62"/>
       <c r="H90" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I90" s="65" t="s">
         <v>14</v>
@@ -12374,7 +12390,7 @@
       </c>
       <c r="G91" s="62"/>
       <c r="H91" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I91" s="65" t="s">
         <v>14</v>
@@ -12403,7 +12419,7 @@
       </c>
       <c r="G92" s="62"/>
       <c r="H92" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I92" s="65" t="s">
         <v>14</v>
@@ -12432,7 +12448,7 @@
       </c>
       <c r="G93" s="62"/>
       <c r="H93" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I93" s="65" t="s">
         <v>14</v>
@@ -12461,7 +12477,7 @@
       </c>
       <c r="G94" s="62"/>
       <c r="H94" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I94" s="65" t="s">
         <v>14</v>
@@ -12490,7 +12506,7 @@
       </c>
       <c r="G95" s="62"/>
       <c r="H95" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I95" s="65" t="s">
         <v>14</v>
@@ -12519,7 +12535,7 @@
       </c>
       <c r="G96" s="62"/>
       <c r="H96" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I96" s="65" t="s">
         <v>14</v>
@@ -12548,7 +12564,7 @@
       </c>
       <c r="G97" s="62"/>
       <c r="H97" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I97" s="65" t="s">
         <v>14</v>
@@ -12577,7 +12593,7 @@
       </c>
       <c r="G98" s="62"/>
       <c r="H98" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I98" s="65" t="s">
         <v>14</v>
@@ -12608,7 +12624,7 @@
         <v>31</v>
       </c>
       <c r="H99" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I99" s="65" t="s">
         <v>14</v>
@@ -12637,7 +12653,7 @@
       </c>
       <c r="G100" s="62"/>
       <c r="H100" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I100" s="65" t="s">
         <v>14</v>
@@ -12666,7 +12682,7 @@
       </c>
       <c r="G101" s="62"/>
       <c r="H101" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I101" s="65" t="s">
         <v>14</v>
@@ -12695,7 +12711,7 @@
       </c>
       <c r="G102" s="62"/>
       <c r="H102" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I102" s="65" t="s">
         <v>14</v>
@@ -12724,7 +12740,7 @@
       </c>
       <c r="G103" s="62"/>
       <c r="H103" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I103" s="65" t="s">
         <v>14</v>
@@ -12753,7 +12769,7 @@
       </c>
       <c r="G104" s="62"/>
       <c r="H104" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I104" s="65" t="s">
         <v>14</v>
@@ -12782,7 +12798,7 @@
       </c>
       <c r="G105" s="62"/>
       <c r="H105" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I105" s="65" t="s">
         <v>14</v>
@@ -12811,7 +12827,7 @@
       </c>
       <c r="G106" s="62"/>
       <c r="H106" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I106" s="65" t="s">
         <v>14</v>
@@ -12840,7 +12856,7 @@
       </c>
       <c r="G107" s="62"/>
       <c r="H107" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I107" s="65" t="s">
         <v>14</v>
@@ -12869,7 +12885,7 @@
       </c>
       <c r="G108" s="62"/>
       <c r="H108" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I108" s="65" t="s">
         <v>14</v>
@@ -12898,7 +12914,7 @@
       </c>
       <c r="G109" s="62"/>
       <c r="H109" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I109" s="65" t="s">
         <v>14</v>
@@ -12927,7 +12943,7 @@
       </c>
       <c r="G110" s="62"/>
       <c r="H110" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I110" s="65" t="s">
         <v>14</v>
@@ -12956,7 +12972,7 @@
       </c>
       <c r="G111" s="62"/>
       <c r="H111" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I111" s="65" t="s">
         <v>14</v>
@@ -12987,7 +13003,7 @@
         <v>112</v>
       </c>
       <c r="H112" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I112" s="65" t="s">
         <v>14</v>
@@ -13016,7 +13032,7 @@
       </c>
       <c r="G113" s="62"/>
       <c r="H113" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I113" s="65" t="s">
         <v>13</v>
@@ -13045,7 +13061,7 @@
       </c>
       <c r="G114" s="62"/>
       <c r="H114" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I114" s="65" t="s">
         <v>14</v>
@@ -13074,7 +13090,7 @@
       </c>
       <c r="G115" s="62"/>
       <c r="H115" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I115" s="65" t="s">
         <v>14</v>
@@ -13103,7 +13119,7 @@
       </c>
       <c r="G116" s="62"/>
       <c r="H116" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I116" s="65" t="s">
         <v>14</v>
@@ -13132,7 +13148,7 @@
       </c>
       <c r="G117" s="62"/>
       <c r="H117" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I117" s="65" t="s">
         <v>14</v>
@@ -13161,7 +13177,7 @@
       </c>
       <c r="G118" s="62"/>
       <c r="H118" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I118" s="65" t="s">
         <v>14</v>
@@ -13190,7 +13206,7 @@
       </c>
       <c r="G119" s="62"/>
       <c r="H119" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I119" s="65" t="s">
         <v>14</v>
@@ -13219,7 +13235,7 @@
       </c>
       <c r="G120" s="62"/>
       <c r="H120" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I120" s="65" t="s">
         <v>14</v>
@@ -13248,7 +13264,7 @@
       </c>
       <c r="G121" s="62"/>
       <c r="H121" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I121" s="65" t="s">
         <v>14</v>
@@ -13277,7 +13293,7 @@
       </c>
       <c r="G122" s="62"/>
       <c r="H122" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I122" s="65" t="s">
         <v>14</v>
@@ -13306,7 +13322,7 @@
       </c>
       <c r="G123" s="62"/>
       <c r="H123" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I123" s="65" t="s">
         <v>13</v>
@@ -13335,7 +13351,7 @@
       </c>
       <c r="G124" s="62"/>
       <c r="H124" s="62" t="s">
-        <v>130</v>
+        <v>370</v>
       </c>
       <c r="I124" s="65" t="s">
         <v>13</v>
@@ -13364,7 +13380,7 @@
       </c>
       <c r="G125" s="62"/>
       <c r="H125" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I125" s="65" t="s">
         <v>13</v>
@@ -13393,7 +13409,7 @@
       </c>
       <c r="G126" s="62"/>
       <c r="H126" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I126" s="65" t="s">
         <v>14</v>
@@ -13422,7 +13438,7 @@
       </c>
       <c r="G127" s="62"/>
       <c r="H127" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I127" s="65" t="s">
         <v>14</v>
@@ -13451,7 +13467,7 @@
       </c>
       <c r="G128" s="62"/>
       <c r="H128" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I128" s="65" t="s">
         <v>14</v>
@@ -13480,7 +13496,7 @@
       </c>
       <c r="G129" s="62"/>
       <c r="H129" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I129" s="65" t="s">
         <v>14</v>
@@ -13509,7 +13525,7 @@
       </c>
       <c r="G130" s="62"/>
       <c r="H130" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I130" s="65" t="s">
         <v>14</v>
@@ -13538,7 +13554,7 @@
       </c>
       <c r="G131" s="62"/>
       <c r="H131" s="62" t="s">
-        <v>135</v>
+        <v>371</v>
       </c>
       <c r="I131" s="65" t="s">
         <v>14</v>
@@ -13567,7 +13583,7 @@
       </c>
       <c r="G132" s="62"/>
       <c r="H132" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I132" s="65" t="s">
         <v>14</v>
@@ -13598,7 +13614,7 @@
         <v>31</v>
       </c>
       <c r="H133" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I133" s="65" t="s">
         <v>14</v>
@@ -13629,7 +13645,7 @@
         <v>31</v>
       </c>
       <c r="H134" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I134" s="65" t="s">
         <v>14</v>
@@ -13658,7 +13674,7 @@
       </c>
       <c r="G135" s="62"/>
       <c r="H135" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I135" s="65" t="s">
         <v>13</v>
@@ -13687,7 +13703,7 @@
       </c>
       <c r="G136" s="62"/>
       <c r="H136" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I136" s="65" t="s">
         <v>14</v>
@@ -13716,7 +13732,7 @@
       </c>
       <c r="G137" s="62"/>
       <c r="H137" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I137" s="65" t="s">
         <v>13</v>
@@ -13745,7 +13761,7 @@
       </c>
       <c r="G138" s="62"/>
       <c r="H138" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I138" s="65" t="s">
         <v>14</v>
@@ -13774,7 +13790,7 @@
       </c>
       <c r="G139" s="62"/>
       <c r="H139" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I139" s="65" t="s">
         <v>13</v>
@@ -13803,7 +13819,7 @@
       </c>
       <c r="G140" s="62"/>
       <c r="H140" s="62" t="s">
-        <v>127</v>
+        <v>368</v>
       </c>
       <c r="I140" s="65" t="s">
         <v>13</v>
@@ -13832,7 +13848,7 @@
       </c>
       <c r="G141" s="62"/>
       <c r="H141" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I141" s="65" t="s">
         <v>14</v>
@@ -13861,7 +13877,7 @@
       </c>
       <c r="G142" s="62"/>
       <c r="H142" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I142" s="65" t="s">
         <v>14</v>
@@ -13890,7 +13906,7 @@
       </c>
       <c r="G143" s="62"/>
       <c r="H143" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I143" s="65" t="s">
         <v>14</v>
@@ -13919,7 +13935,7 @@
       </c>
       <c r="G144" s="62"/>
       <c r="H144" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I144" s="65" t="s">
         <v>14</v>
@@ -13948,7 +13964,7 @@
       </c>
       <c r="G145" s="62"/>
       <c r="H145" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I145" s="65" t="s">
         <v>14</v>
@@ -13977,7 +13993,7 @@
       </c>
       <c r="G146" s="62"/>
       <c r="H146" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I146" s="65" t="s">
         <v>14</v>
@@ -14006,7 +14022,7 @@
       </c>
       <c r="G147" s="62"/>
       <c r="H147" s="62" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="I147" s="65" t="s">
         <v>14</v>
@@ -14035,7 +14051,7 @@
       </c>
       <c r="G148" s="62"/>
       <c r="H148" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I148" s="65" t="s">
         <v>74</v>
@@ -14064,7 +14080,7 @@
       </c>
       <c r="G149" s="62"/>
       <c r="H149" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I149" s="65" t="s">
         <v>74</v>
@@ -14093,7 +14109,7 @@
       </c>
       <c r="G150" s="62"/>
       <c r="H150" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I150" s="65" t="s">
         <v>74</v>
@@ -14122,7 +14138,7 @@
       </c>
       <c r="G151" s="62"/>
       <c r="H151" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I151" s="65" t="s">
         <v>74</v>
@@ -14151,7 +14167,7 @@
       </c>
       <c r="G152" s="62"/>
       <c r="H152" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I152" s="65" t="s">
         <v>13</v>
@@ -14180,7 +14196,7 @@
       </c>
       <c r="G153" s="62"/>
       <c r="H153" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I153" s="65" t="s">
         <v>14</v>
@@ -14211,7 +14227,7 @@
         <v>31</v>
       </c>
       <c r="H154" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I154" s="65" t="s">
         <v>14</v>
@@ -14240,7 +14256,7 @@
       </c>
       <c r="G155" s="62"/>
       <c r="H155" s="62" t="s">
-        <v>164</v>
+        <v>368</v>
       </c>
       <c r="I155" s="65" t="s">
         <v>14</v>
@@ -14269,7 +14285,7 @@
       </c>
       <c r="G156" s="62"/>
       <c r="H156" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I156" s="65" t="s">
         <v>14</v>
@@ -14298,7 +14314,7 @@
       </c>
       <c r="G157" s="62"/>
       <c r="H157" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I157" s="65" t="s">
         <v>14</v>
@@ -14327,7 +14343,7 @@
       </c>
       <c r="G158" s="62"/>
       <c r="H158" s="62" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I158" s="65" t="s">
         <v>14</v>
@@ -14356,7 +14372,7 @@
       </c>
       <c r="G159" s="62"/>
       <c r="H159" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I159" s="65" t="s">
         <v>14</v>
@@ -14385,7 +14401,7 @@
       </c>
       <c r="G160" s="63"/>
       <c r="H160" s="141" t="s">
-        <v>164</v>
+        <v>368</v>
       </c>
       <c r="I160" s="140" t="s">
         <v>14</v>
@@ -14413,7 +14429,7 @@
         <v>199</v>
       </c>
       <c r="H161" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I161" s="143" t="s">
         <v>14</v>
@@ -14443,7 +14459,7 @@
         <v>197</v>
       </c>
       <c r="H162" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I162" s="143" t="s">
         <v>14</v>
@@ -14473,7 +14489,7 @@
         <v>195</v>
       </c>
       <c r="H163" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I163" s="143" t="s">
         <v>14</v>
@@ -14503,7 +14519,7 @@
         <v>193</v>
       </c>
       <c r="H164" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I164" s="143" t="s">
         <v>14</v>
@@ -14533,7 +14549,7 @@
         <v>191</v>
       </c>
       <c r="H165" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I165" s="150" t="s">
         <v>13</v>
@@ -14563,7 +14579,7 @@
         <v>188</v>
       </c>
       <c r="H166" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I166" s="143" t="s">
         <v>14</v>
@@ -14593,7 +14609,7 @@
         <v>205</v>
       </c>
       <c r="H167" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I167" s="150" t="s">
         <v>13</v>
@@ -14623,7 +14639,7 @@
         <v>203</v>
       </c>
       <c r="H168" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I168" s="150" t="s">
         <v>13</v>
@@ -14653,7 +14669,7 @@
         <v>3169</v>
       </c>
       <c r="H169" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I169" s="150" t="s">
         <v>14</v>
@@ -14683,7 +14699,7 @@
         <v>4149</v>
       </c>
       <c r="H170" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I170" s="150" t="s">
         <v>14</v>
@@ -14713,7 +14729,7 @@
         <v>5077</v>
       </c>
       <c r="H171" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I171" s="150" t="s">
         <v>14</v>
@@ -14743,7 +14759,7 @@
         <v>1378</v>
       </c>
       <c r="H172" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I172" s="150" t="s">
         <v>13</v>
@@ -14773,7 +14789,7 @@
         <v>1086</v>
       </c>
       <c r="H173" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I173" s="150" t="s">
         <v>14</v>
@@ -14803,7 +14819,7 @@
         <v>1079</v>
       </c>
       <c r="H174" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I174" s="150" t="s">
         <v>13</v>
@@ -14833,7 +14849,7 @@
         <v>1086</v>
       </c>
       <c r="H175" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I175" s="150" t="s">
         <v>13</v>
@@ -14863,7 +14879,7 @@
         <v>2104</v>
       </c>
       <c r="H176" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I176" s="150" t="s">
         <v>14</v>
@@ -14893,7 +14909,7 @@
         <v>1063</v>
       </c>
       <c r="H177" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I177" s="150" t="s">
         <v>14</v>
@@ -14923,7 +14939,7 @@
         <v>223</v>
       </c>
       <c r="H178" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I178" s="150" t="s">
         <v>14</v>
@@ -14953,7 +14969,7 @@
         <v>224</v>
       </c>
       <c r="H179" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I179" s="150" t="s">
         <v>14</v>
@@ -14983,7 +14999,7 @@
         <v>2373</v>
       </c>
       <c r="H180" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I180" s="150" t="s">
         <v>14</v>
@@ -15013,7 +15029,7 @@
         <v>3281</v>
       </c>
       <c r="H181" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I181" s="150" t="s">
         <v>14</v>
@@ -15043,7 +15059,7 @@
         <v>4260</v>
       </c>
       <c r="H182" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I182" s="150" t="s">
         <v>14</v>
@@ -15073,7 +15089,7 @@
         <v>225</v>
       </c>
       <c r="H183" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I183" s="150" t="s">
         <v>14</v>
@@ -15106,7 +15122,7 @@
         <v>31</v>
       </c>
       <c r="H184" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I184" s="150" t="s">
         <v>14</v>
@@ -15136,7 +15152,7 @@
         <v>230</v>
       </c>
       <c r="H185" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I185" s="150" t="s">
         <v>14</v>
@@ -15166,7 +15182,7 @@
         <v>1685</v>
       </c>
       <c r="H186" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I186" s="150" t="s">
         <v>14</v>
@@ -15196,7 +15212,7 @@
         <v>232</v>
       </c>
       <c r="H187" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I187" s="150" t="s">
         <v>14</v>
@@ -15226,7 +15242,7 @@
         <v>234</v>
       </c>
       <c r="H188" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I188" s="150" t="s">
         <v>14</v>
@@ -15256,7 +15272,7 @@
         <v>235</v>
       </c>
       <c r="H189" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I189" s="150" t="s">
         <v>14</v>
@@ -15286,7 +15302,7 @@
         <v>1118</v>
       </c>
       <c r="H190" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I190" s="150" t="s">
         <v>14</v>
@@ -15316,7 +15332,7 @@
         <v>237</v>
       </c>
       <c r="H191" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I191" s="150" t="s">
         <v>14</v>
@@ -15346,7 +15362,7 @@
         <v>2186</v>
       </c>
       <c r="H192" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I192" s="150" t="s">
         <v>14</v>
@@ -15376,7 +15392,7 @@
         <v>239</v>
       </c>
       <c r="H193" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I193" s="150" t="s">
         <v>14</v>
@@ -15406,7 +15422,7 @@
         <v>240</v>
       </c>
       <c r="H194" s="147" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="I194" s="150" t="s">
         <v>14</v>
@@ -15439,7 +15455,7 @@
         <v>31</v>
       </c>
       <c r="H195" s="62" t="s">
-        <v>32</v>
+        <v>369</v>
       </c>
       <c r="I195" s="150" t="s">
         <v>14</v>
@@ -15472,7 +15488,7 @@
         <v>112</v>
       </c>
       <c r="H196" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I196" s="150" t="s">
         <v>14</v>
@@ -15505,7 +15521,7 @@
         <v>112</v>
       </c>
       <c r="H197" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I197" s="150" t="s">
         <v>14</v>
@@ -15538,7 +15554,7 @@
         <v>112</v>
       </c>
       <c r="H198" s="62" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I198" s="150" t="s">
         <v>14</v>
@@ -15568,7 +15584,7 @@
         <v>3220</v>
       </c>
       <c r="H199" s="147" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I199" s="150" t="s">
         <v>14</v>
@@ -15598,7 +15614,7 @@
         <v>5334</v>
       </c>
       <c r="H200" s="155" t="s">
-        <v>19</v>
+        <v>367</v>
       </c>
       <c r="I200" s="156" t="s">
         <v>14</v>
@@ -15627,32 +15643,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -15663,13 +15679,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
@@ -15974,31 +15990,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -16009,13 +16025,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="17" t="s">
         <v>7</v>
       </c>
@@ -16268,31 +16284,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="181" t="s">
         <v>168</v>
       </c>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="171" t="s">
+      <c r="C5" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="172"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="177" t="s">
+      <c r="D5" s="183"/>
+      <c r="E5" s="184"/>
+      <c r="F5" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="177" t="s">
+      <c r="G5" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -16303,13 +16319,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="174"/>
-      <c r="D6" s="175"/>
-      <c r="E6" s="176"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="178"/>
+      <c r="A6" s="180"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="185"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="189"/>
+      <c r="G6" s="189"/>
       <c r="H6" s="17" t="s">
         <v>7</v>
       </c>
@@ -16540,29 +16556,29 @@
       </c>
     </row>
     <row r="15" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="182" t="s">
+      <c r="A15" s="168" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="183">
+      <c r="B15" s="169">
         <v>9</v>
       </c>
-      <c r="C15" s="184" t="s">
+      <c r="C15" s="170" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="184" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="184">
+      <c r="D15" s="170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="170">
         <v>5178</v>
       </c>
-      <c r="F15" s="184"/>
-      <c r="G15" s="184" t="s">
+      <c r="F15" s="170"/>
+      <c r="G15" s="170" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="190" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="191" t="s">
+      <c r="H15" s="176" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="177" t="s">
         <v>14</v>
       </c>
     </row>
@@ -16594,29 +16610,29 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="182" t="s">
+      <c r="A17" s="168" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="183">
+      <c r="B17" s="169">
         <v>11</v>
       </c>
-      <c r="C17" s="184" t="s">
+      <c r="C17" s="170" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="184" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="184" t="s">
+      <c r="D17" s="170" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="170" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="184"/>
-      <c r="G17" s="184" t="s">
+      <c r="F17" s="170"/>
+      <c r="G17" s="170" t="s">
         <v>19</v>
       </c>
-      <c r="H17" s="190" t="s">
-        <v>14</v>
-      </c>
-      <c r="I17" s="191" t="s">
+      <c r="H17" s="176" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="177" t="s">
         <v>14</v>
       </c>
     </row>
@@ -16787,33 +16803,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="179" t="s">
+      <c r="B1" s="190" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
+      <c r="C1" s="190"/>
+      <c r="D1" s="190"/>
+      <c r="E1" s="190"/>
+      <c r="F1" s="190"/>
+      <c r="G1" s="190"/>
+      <c r="H1" s="190"/>
+      <c r="I1" s="190"/>
     </row>
     <row r="2" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="168" t="s">
+      <c r="A2" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="171" t="s">
+      <c r="C2" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="172"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="177" t="s">
+      <c r="D2" s="183"/>
+      <c r="E2" s="184"/>
+      <c r="F2" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="177" t="s">
+      <c r="G2" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H2" s="24" t="s">
@@ -16827,13 +16843,13 @@
       <c r="L2" s="25"/>
     </row>
     <row r="3" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="169"/>
-      <c r="B3" s="169"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
+      <c r="A3" s="180"/>
+      <c r="B3" s="180"/>
+      <c r="C3" s="185"/>
+      <c r="D3" s="186"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
       <c r="H3" s="26" t="s">
         <v>7</v>
       </c>
@@ -17176,33 +17192,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="179" t="s">
+      <c r="B1" s="190" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
+      <c r="C1" s="190"/>
+      <c r="D1" s="190"/>
+      <c r="E1" s="190"/>
+      <c r="F1" s="190"/>
+      <c r="G1" s="190"/>
+      <c r="H1" s="190"/>
+      <c r="I1" s="190"/>
     </row>
     <row r="2" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="168" t="s">
+      <c r="A2" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="171" t="s">
+      <c r="C2" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="172"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="177" t="s">
+      <c r="D2" s="183"/>
+      <c r="E2" s="184"/>
+      <c r="F2" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="177" t="s">
+      <c r="G2" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H2" s="52" t="s">
@@ -17216,13 +17232,13 @@
       <c r="L2" s="25"/>
     </row>
     <row r="3" spans="1:12" s="1" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="169"/>
-      <c r="B3" s="169"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
+      <c r="A3" s="180"/>
+      <c r="B3" s="180"/>
+      <c r="C3" s="185"/>
+      <c r="D3" s="186"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
       <c r="H3" s="52" t="s">
         <v>7</v>
       </c>
@@ -17624,26 +17640,26 @@
       <c r="L16" s="25"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="180" t="s">
+      <c r="B18" s="191" t="s">
         <v>175</v>
       </c>
-      <c r="C18" s="180"/>
-      <c r="D18" s="180"/>
-      <c r="E18" s="180"/>
-      <c r="F18" s="180"/>
-      <c r="G18" s="180"/>
-      <c r="H18" s="180"/>
-      <c r="I18" s="180"/>
+      <c r="C18" s="191"/>
+      <c r="D18" s="191"/>
+      <c r="E18" s="191"/>
+      <c r="F18" s="191"/>
+      <c r="G18" s="191"/>
+      <c r="H18" s="191"/>
+      <c r="I18" s="191"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="180"/>
-      <c r="C19" s="180"/>
-      <c r="D19" s="180"/>
-      <c r="E19" s="180"/>
-      <c r="F19" s="180"/>
-      <c r="G19" s="180"/>
-      <c r="H19" s="180"/>
-      <c r="I19" s="180"/>
+      <c r="B19" s="191"/>
+      <c r="C19" s="191"/>
+      <c r="D19" s="191"/>
+      <c r="E19" s="191"/>
+      <c r="F19" s="191"/>
+      <c r="G19" s="191"/>
+      <c r="H19" s="191"/>
+      <c r="I19" s="191"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -17674,33 +17690,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="B1" s="179" t="s">
+      <c r="B1" s="190" t="s">
         <v>176</v>
       </c>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
+      <c r="C1" s="190"/>
+      <c r="D1" s="190"/>
+      <c r="E1" s="190"/>
+      <c r="F1" s="190"/>
+      <c r="G1" s="190"/>
+      <c r="H1" s="190"/>
+      <c r="I1" s="190"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="168" t="s">
+      <c r="A2" s="179" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="171" t="s">
+      <c r="C2" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="172"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="177" t="s">
+      <c r="D2" s="183"/>
+      <c r="E2" s="184"/>
+      <c r="F2" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="177" t="s">
+      <c r="G2" s="188" t="s">
         <v>4</v>
       </c>
       <c r="H2" s="53" t="s">
@@ -17711,13 +17727,13 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="169"/>
-      <c r="B3" s="169"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
+      <c r="A3" s="180"/>
+      <c r="B3" s="180"/>
+      <c r="C3" s="185"/>
+      <c r="D3" s="186"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
       <c r="H3" s="52" t="s">
         <v>7</v>
       </c>
@@ -17969,26 +17985,26 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="180" t="s">
+      <c r="B14" s="191" t="s">
         <v>177</v>
       </c>
-      <c r="C14" s="180"/>
-      <c r="D14" s="180"/>
-      <c r="E14" s="180"/>
-      <c r="F14" s="180"/>
-      <c r="G14" s="180"/>
-      <c r="H14" s="180"/>
-      <c r="I14" s="180"/>
+      <c r="C14" s="191"/>
+      <c r="D14" s="191"/>
+      <c r="E14" s="191"/>
+      <c r="F14" s="191"/>
+      <c r="G14" s="191"/>
+      <c r="H14" s="191"/>
+      <c r="I14" s="191"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="180"/>
-      <c r="C15" s="180"/>
-      <c r="D15" s="180"/>
-      <c r="E15" s="180"/>
-      <c r="F15" s="180"/>
-      <c r="G15" s="180"/>
-      <c r="H15" s="180"/>
-      <c r="I15" s="180"/>
+      <c r="B15" s="191"/>
+      <c r="C15" s="191"/>
+      <c r="D15" s="191"/>
+      <c r="E15" s="191"/>
+      <c r="F15" s="191"/>
+      <c r="G15" s="191"/>
+      <c r="H15" s="191"/>
+      <c r="I15" s="191"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>